<commit_message>
all websites requested 2025-06-13 done
</commit_message>
<xml_diff>
--- a/storage_results.xlsx
+++ b/storage_results.xlsx
@@ -10,6 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-06-18_sopris_results" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-06-18_storquest_results" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-06-18_storage_mart_results" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-06-18_all_hours_results" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-06-18_carbondale_results" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1829,4 +1831,656 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>unit_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Standard (5 x 5 x 4)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>$79</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Standard (5 x 5)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>$99</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>5X5CC (5 x 5 x 8)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>$117</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Standard (5 x 10)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>$175</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5X10CC (5 x 10)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>$190</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10X10CC (10 x 10)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>$270</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Standard (10 x 15)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>$375</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Standard (10 x 20)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>$450</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Heated 10X20CC (10 x 20)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>$500</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Standard (10 x 25)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>$575</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Standard (10 x 30)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>$695</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Standard (15 x 30)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>$760</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Standard (20 x 20)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>$750</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Paved Outside Parking (19 x 9)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>$199</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ultimate 10 x 10 (10 x 10 x 10)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>$299</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ultimate  (10 x 20 x 10)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>$579</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ultimate 10 x 30 (10 x 30 x 10)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>$650</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ultimate 10 x 40 (10 x 40 x 10)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>$1,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ultimate 20 x 40 (20 x 40 x 10)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>$1,737</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Ultimate 10 x 10 (10 x 10 x 10)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>$299</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ultimate 10 x 20 (10 x 20 x 10)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>$579</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ultimate 10 x 30 (30 x 10)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>$650</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ultimate 20 x 20  (20 x 20 x 10)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>$725</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>unit_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>10X20</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>$365.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10x10</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>$199.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>10x10</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>$199.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>10x10</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>$260.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>10x15</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>$240.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10x15</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>$305.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>10x20</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>$365.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>10x25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>$405.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>10x30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>$475.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>10x30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>$450.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>12x20</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>$385.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>12x20</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>$440.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12x30 (CC)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>$570.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>12x35</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>$470.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>13x25</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>$440.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>15x20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>$440.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>15x25</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>$530.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>3X2.7</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>$50.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>5X4X4</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>$80.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>5X5X4</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>$85.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>5X5X8</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>$90.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>5x10</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>$165.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>5x10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>$175.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>5x10</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>$175.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>7x25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>$260.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Outdoor Parking</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>$110.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Outdoor Parking</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>$145.00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
working with task scheduler
</commit_message>
<xml_diff>
--- a/storage_results.xlsx
+++ b/storage_results.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-06-30_sopris_results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-06-30_storquest_results" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-06-30_storage_mart_results" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-06-30_all_hours_results" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-06-30_carbondale_results" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-06-30_basalt_results" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-01 Sopris Self Storage" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-01 StorQuest Self Storage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-01 StorageMart" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-01 All Hours Storage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-01 Carbondale Mini Storage" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-01 Basalt Mini Storage" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +449,16 @@
           <t>price</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>climate_controlled</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -466,6 +476,14 @@
           <t>85.00</t>
         </is>
       </c>
+      <c r="D2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -483,6 +501,14 @@
           <t>87.00</t>
         </is>
       </c>
+      <c r="D3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -500,6 +526,14 @@
           <t>95.00</t>
         </is>
       </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -517,6 +551,14 @@
           <t>95.00</t>
         </is>
       </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -534,6 +576,14 @@
           <t>95.00</t>
         </is>
       </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>tier 1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -551,6 +601,14 @@
           <t>139.00</t>
         </is>
       </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -568,6 +626,14 @@
           <t>153.00</t>
         </is>
       </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -577,70 +643,102 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Indoor Good 2nd floor</t>
+          <t>Indoor Good 1st floor</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>153.00</t>
+        </is>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5x10</t>
+          <t>10x5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Indoor Good 3rd floor</t>
+          <t>Indoor Good 2nd floor</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>159.00</t>
+          <t>153.00</t>
+        </is>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8x9</t>
+          <t>5x10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bins Self Storage</t>
+          <t>Indoor Good 3rd floor</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>166.00</t>
+          <t>159.00</t>
+        </is>
+      </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>10x20</t>
+          <t>8x9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Indoor Good 3rd floor</t>
+          <t>Bins Self Storage</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>170.00</t>
+          <t>166.00</t>
+        </is>
+      </c>
+      <c r="D12" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>10x21</t>
+          <t>10x20</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -651,30 +749,46 @@
       <c r="C13" t="inlineStr">
         <is>
           <t>170.00</t>
+        </is>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>10x20</t>
+          <t>10x21</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Indoor Better 3rd floor</t>
+          <t>Indoor Good 3rd floor</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>173.00</t>
+          <t>170.00</t>
+        </is>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10x21</t>
+          <t>10x20</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -685,40 +799,64 @@
       <c r="C15" t="inlineStr">
         <is>
           <t>173.00</t>
+        </is>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>tier 2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>15x5</t>
+          <t>10x21</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Indoor Good 2nd floor</t>
+          <t>Indoor Better 3rd floor</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>175.00</t>
+          <t>173.00</t>
+        </is>
+      </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>tier 2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10x20</t>
+          <t>15x5</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Indoor Best 3rd floor</t>
+          <t>Indoor Good 2nd floor</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>175.00</t>
+        </is>
+      </c>
+      <c r="D17" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
@@ -738,21 +876,37 @@
           <t>176.00</t>
         </is>
       </c>
+      <c r="D18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10x10</t>
+          <t>10x20</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Indoor Good 2nd floor</t>
+          <t>Indoor Best 3rd floor</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>212.00</t>
+          <t>181.00</t>
+        </is>
+      </c>
+      <c r="D19" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>tier 3</t>
         </is>
       </c>
     </row>
@@ -764,29 +918,45 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Indoor Good 3rd floor</t>
+          <t>Indoor Good 2nd floor</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>212.00</t>
+        </is>
+      </c>
+      <c r="D20" t="b">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10x11</t>
+          <t>10x10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Indoor Good 2nd floor</t>
+          <t>Indoor Good 3rd floor</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>212.00</t>
+        </is>
+      </c>
+      <c r="D21" t="b">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
@@ -798,29 +968,45 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Indoor Good 3rd floor</t>
+          <t>Indoor Good 2nd floor</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>212.00</t>
+        </is>
+      </c>
+      <c r="D22" t="b">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10x10</t>
+          <t>10x11</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Indoor Better 2nd floor</t>
+          <t>Indoor Good 3rd floor</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215.00</t>
+          <t>212.00</t>
+        </is>
+      </c>
+      <c r="D23" t="b">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
@@ -832,19 +1018,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Indoor Better 3rd floor</t>
+          <t>DriveUp Original Units</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>215.00</t>
+        </is>
+      </c>
+      <c r="D24" t="b">
+        <v>0</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>10x11</t>
+          <t>10x10</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -855,6 +1049,14 @@
       <c r="C25" t="inlineStr">
         <is>
           <t>215.00</t>
+        </is>
+      </c>
+      <c r="D25" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>tier 2</t>
         </is>
       </c>
     </row>
@@ -866,63 +1068,95 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DriveUp Original Units</t>
+          <t>Indoor Better 3rd floor</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>219.00</t>
+          <t>215.00</t>
+        </is>
+      </c>
+      <c r="D26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>tier 2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>10x10</t>
+          <t>10x11</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Indoor Good 1st floor</t>
+          <t>Indoor Better 2nd floor</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>220.00</t>
+          <t>215.00</t>
+        </is>
+      </c>
+      <c r="D27" t="b">
+        <v>1</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>tier 2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>10x15</t>
+          <t>10x10</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Indoor Good 2nd floor</t>
+          <t>Indoor Best 2nd floor</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>270.00</t>
+          <t>219.00</t>
+        </is>
+      </c>
+      <c r="D28" t="b">
+        <v>1</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>tier 3</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>10x15</t>
+          <t>10x10</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Indoor Good 3rd floor</t>
+          <t>Indoor Good 1st floor</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>270.00</t>
+          <t>220.00</t>
+        </is>
+      </c>
+      <c r="D29" t="b">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
@@ -934,29 +1168,45 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Indoor Good 1st floor</t>
+          <t>Indoor Good 2nd floor</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>309.00</t>
+          <t>270.00</t>
+        </is>
+      </c>
+      <c r="D30" t="b">
+        <v>1</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>10x16</t>
+          <t>10x15</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Indoor Good 1st floor</t>
+          <t>Indoor Good 3rd floor</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>320.00</t>
+          <t>270.00</t>
+        </is>
+      </c>
+      <c r="D31" t="b">
+        <v>1</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
@@ -968,46 +1218,70 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Indoor Best 1st floor</t>
+          <t>Indoor Better 2nd floor</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>324.00</t>
+          <t>278.00</t>
+        </is>
+      </c>
+      <c r="D32" t="b">
+        <v>1</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>tier 2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>10x16</t>
+          <t>10x15</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Indoor Better 1st floor</t>
+          <t>Indoor Good 1st floor</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>338.00</t>
+          <t>312.00</t>
+        </is>
+      </c>
+      <c r="D33" t="b">
+        <v>1</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>10x20</t>
+          <t>10x16</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DriveUp Original Units</t>
+          <t>Indoor Good 1st floor</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>340.00</t>
+          <t>320.00</t>
+        </is>
+      </c>
+      <c r="D34" t="b">
+        <v>1</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
@@ -1019,19 +1293,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Indoor Good 2nd floor</t>
+          <t>DriveUp Original Units</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>340.00</t>
+          <t>337.00</t>
+        </is>
+      </c>
+      <c r="D35" t="b">
+        <v>0</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>10x21</t>
+          <t>10x20</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1042,30 +1324,46 @@
       <c r="C36" t="inlineStr">
         <is>
           <t>340.00</t>
+        </is>
+      </c>
+      <c r="D36" t="b">
+        <v>1</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>10x20</t>
+          <t>10x21</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Indoor Better 2nd floor</t>
+          <t>Indoor Good 2nd floor</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>345.00</t>
+          <t>340.00</t>
+        </is>
+      </c>
+      <c r="D37" t="b">
+        <v>1</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>10x21</t>
+          <t>10x20</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1076,30 +1374,46 @@
       <c r="C38" t="inlineStr">
         <is>
           <t>345.00</t>
+        </is>
+      </c>
+      <c r="D38" t="b">
+        <v>1</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>tier 2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>10x20</t>
+          <t>10x21</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Indoor Best 2nd floor</t>
+          <t>Indoor Better 2nd floor</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>350.00</t>
+          <t>345.00</t>
+        </is>
+      </c>
+      <c r="D39" t="b">
+        <v>1</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>tier 2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>10x21</t>
+          <t>10x20</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1110,91 +1424,189 @@
       <c r="C40" t="inlineStr">
         <is>
           <t>350.00</t>
+        </is>
+      </c>
+      <c r="D40" t="b">
+        <v>1</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>tier 3</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>10x20</t>
+          <t>10x21</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Indoor Better 1st floor</t>
+          <t>Indoor Best 2nd floor</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>410.00</t>
+          <t>350.00</t>
+        </is>
+      </c>
+      <c r="D41" t="b">
+        <v>1</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>tier 3</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>13.5x18.5</t>
+          <t>10x20</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1201 Bldg</t>
+          <t>Indoor Better 1st floor</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
           <t>410.00</t>
+        </is>
+      </c>
+      <c r="D42" t="b">
+        <v>1</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>tier 2</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>10x20</t>
+          <t>13.5x18.5</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Indoor Best 1st floor</t>
+          <t>1201 Bldg</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>420.00</t>
+          <t>410.00</t>
+        </is>
+      </c>
+      <c r="D43" t="b">
+        <v>0</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>10x25</t>
+          <t>10x20</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Driveup New</t>
+          <t>Indoor Best 1st floor</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>599.00</t>
+          <t>420.00</t>
+        </is>
+      </c>
+      <c r="D44" t="b">
+        <v>1</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>tier 3</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>12.5x22</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Indoor Good 1st floor</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>550.00</t>
+        </is>
+      </c>
+      <c r="D45" t="b">
+        <v>1</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>tier 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>10x25</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Driveup New</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>599.00</t>
+        </is>
+      </c>
+      <c r="D46" t="b">
+        <v>0</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>10x30</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>Driveup New</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>749.00</t>
+        </is>
+      </c>
+      <c r="D47" t="b">
+        <v>0</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1228,6 +1640,16 @@
           <t>price</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>climate_controlled</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1245,6 +1667,14 @@
           <t>88.00</t>
         </is>
       </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1262,6 +1692,14 @@
           <t>101.00</t>
         </is>
       </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1279,6 +1717,14 @@
           <t>181.00</t>
         </is>
       </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1296,6 +1742,14 @@
           <t>190.00</t>
         </is>
       </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1313,6 +1767,14 @@
           <t>293.00</t>
         </is>
       </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1330,11 +1792,19 @@
           <t>228.00</t>
         </is>
       </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>8x15</t>
+          <t>10x10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1344,31 +1814,47 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>273.00</t>
+          <t>239.00</t>
+        </is>
+      </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10x13</t>
+          <t>8x15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Elevator AccessClimate Controlled</t>
+          <t>1st FloorClimate Controlled</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>233.00</t>
+          <t>273.00</t>
+        </is>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>10x15</t>
+          <t>10x13</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1378,58 +1864,90 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>259.00</t>
+          <t>233.00</t>
+        </is>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9x18</t>
+          <t>10x15</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Elevator AccessPremiumClimate Controlled</t>
+          <t>Elevator AccessClimate Controlled</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>376.00</t>
+          <t>259.00</t>
+        </is>
+      </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>10x17</t>
+          <t>9x18</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Drive Up Access</t>
+          <t>Elevator AccessPremiumClimate Controlled</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>384.00</t>
+          <t>376.00</t>
+        </is>
+      </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>tier 3</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>9x19</t>
+          <t>10x17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Elevator AccessClimate Controlled</t>
+          <t>Drive Up Access</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>389.00</t>
+          <t>384.00</t>
+        </is>
+      </c>
+      <c r="D13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
@@ -1446,14 +1964,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>449.00</t>
+          <t>376.00</t>
+        </is>
+      </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10x18</t>
+          <t>9x19</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1463,7 +1989,15 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>386.00</t>
+          <t>389.00</t>
+        </is>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
@@ -1475,12 +2009,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1st FloorClimate Controlled</t>
+          <t>Elevator AccessClimate Controlled</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>410.00</t>
+          <t>386.00</t>
+        </is>
+      </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
@@ -1497,24 +2039,40 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>467.00</t>
+          <t>397.00</t>
+        </is>
+      </c>
+      <c r="D17" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10x20</t>
+          <t>10x18</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Elevator AccessClimate Controlled</t>
+          <t>1st FloorClimate Controlled</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>429.00</t>
+          <t>410.00</t>
+        </is>
+      </c>
+      <c r="D18" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
@@ -1526,12 +2084,45 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>Elevator AccessClimate Controlled</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>429.00</t>
+        </is>
+      </c>
+      <c r="D19" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10x20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>Drive Up Access</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>514.00</t>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>441.00</t>
+        </is>
+      </c>
+      <c r="D20" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
@@ -1546,7 +2137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1565,6 +2156,16 @@
           <t>price</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>climate_controlled</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1582,38 +2183,62 @@
           <t>104.00</t>
         </is>
       </c>
+      <c r="D2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5X5X8</t>
+          <t>5X10X8</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Indoor First Floor Access Non-Climate Control</t>
+          <t>Drive-Up Non-Climate Control</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>114.00</t>
+          <t>174.00</t>
+        </is>
+      </c>
+      <c r="D3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>5X10X8</t>
+          <t>5X5X8</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Drive-Up Non-Climate Control</t>
+          <t>Indoor Heated First Floor Access</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>174.00</t>
+          <t>197.00</t>
+        </is>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
@@ -1633,6 +2258,14 @@
           <t>234.00</t>
         </is>
       </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1650,6 +2283,14 @@
           <t>257.00</t>
         </is>
       </c>
+      <c r="D6" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1667,6 +2308,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1684,6 +2333,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1701,6 +2358,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D9" t="b">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1718,38 +2383,62 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5X5X8</t>
+          <t>5X8X8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Indoor Heated First Floor Access A/C &amp; Heat</t>
+          <t>Indoor First Floor Access A/C &amp; Heat</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>Sold Out</t>
+        </is>
+      </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5X8X8</t>
+          <t>5X5X8</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Indoor First Floor Access A/C &amp; Heat</t>
+          <t>Indoor First Floor Access Non-Climate Control</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>Sold Out</t>
+        </is>
+      </c>
+      <c r="D12" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
@@ -1769,6 +2458,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1786,6 +2483,14 @@
           <t>259.00</t>
         </is>
       </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1803,6 +2508,14 @@
           <t>364.00</t>
         </is>
       </c>
+      <c r="D15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1820,6 +2533,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1837,6 +2558,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D17" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1854,6 +2583,14 @@
           <t>449.00</t>
         </is>
       </c>
+      <c r="D18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1871,6 +2608,14 @@
           <t>629.00</t>
         </is>
       </c>
+      <c r="D19" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1888,6 +2633,14 @@
           <t>902.00</t>
         </is>
       </c>
+      <c r="D20" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1905,6 +2658,14 @@
           <t>1019.00</t>
         </is>
       </c>
+      <c r="D21" t="b">
+        <v>0</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1922,6 +2683,14 @@
           <t>1132.00</t>
         </is>
       </c>
+      <c r="D22" t="b">
+        <v>0</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1939,6 +2708,14 @@
           <t>1254.00</t>
         </is>
       </c>
+      <c r="D23" t="b">
+        <v>0</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1956,6 +2733,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D24" t="b">
+        <v>0</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1973,6 +2758,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D25" t="b">
+        <v>0</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1990,6 +2783,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2007,6 +2808,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D27" t="b">
+        <v>0</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2024,6 +2833,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D28" t="b">
+        <v>0</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2041,6 +2858,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D29" t="b">
+        <v>0</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2058,6 +2883,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D30" t="b">
+        <v>0</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2075,6 +2908,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D31" t="b">
+        <v>1</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2092,6 +2933,14 @@
           <t>159.00</t>
         </is>
       </c>
+      <c r="D32" t="b">
+        <v>0</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2109,6 +2958,14 @@
           <t>169.00</t>
         </is>
       </c>
+      <c r="D33" t="b">
+        <v>0</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2126,6 +2983,14 @@
           <t>179.00</t>
         </is>
       </c>
+      <c r="D34" t="b">
+        <v>0</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2143,130 +3008,194 @@
           <t>199.00</t>
         </is>
       </c>
+      <c r="D35" t="b">
+        <v>0</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>8X38</t>
+          <t>10X23</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Non-Paved</t>
+          <t>Seasonal Non-Paved</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>229.00</t>
+          <t>209.00</t>
+        </is>
+      </c>
+      <c r="D36" t="b">
+        <v>0</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>8X33</t>
+          <t>8X28</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Seasonal Paved</t>
+          <t>Paved</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>244.00</t>
+          <t>228.00</t>
+        </is>
+      </c>
+      <c r="D37" t="b">
+        <v>0</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>10X28</t>
+          <t>8X38</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Paved</t>
+          <t>Non-Paved</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>259.00</t>
+          <t>229.00</t>
+        </is>
+      </c>
+      <c r="D38" t="b">
+        <v>0</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>10X18</t>
+          <t>8X33</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Non-Paved</t>
+          <t>Seasonal Paved</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Sold Out</t>
+          <t>244.00</t>
+        </is>
+      </c>
+      <c r="D39" t="b">
+        <v>0</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>10X23</t>
+          <t>10X28</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Seasonal Non-Paved</t>
+          <t>Paved</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Sold Out</t>
+          <t>259.00</t>
+        </is>
+      </c>
+      <c r="D40" t="b">
+        <v>0</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>10X23</t>
+          <t>10X18</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Paved</t>
+          <t>Non-Paved</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
           <t>Sold Out</t>
+        </is>
+      </c>
+      <c r="D41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>10X33</t>
+          <t>10X23</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Non-Paved</t>
+          <t>Paved</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
           <t>Sold Out</t>
+        </is>
+      </c>
+      <c r="D42" t="b">
+        <v>0</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>8X17</t>
+          <t>10X33</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2277,13 +3206,21 @@
       <c r="C43" t="inlineStr">
         <is>
           <t>Sold Out</t>
+        </is>
+      </c>
+      <c r="D43" t="b">
+        <v>0</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>8X21</t>
+          <t>8X17</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2294,23 +3231,39 @@
       <c r="C44" t="inlineStr">
         <is>
           <t>Sold Out</t>
+        </is>
+      </c>
+      <c r="D44" t="b">
+        <v>0</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>8X28</t>
+          <t>8X21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Paved</t>
+          <t>Non-Paved</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
           <t>Sold Out</t>
+        </is>
+      </c>
+      <c r="D45" t="b">
+        <v>0</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
@@ -2330,6 +3283,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D46" t="b">
+        <v>0</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2347,6 +3308,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D47" t="b">
+        <v>0</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2364,6 +3333,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D48" t="b">
+        <v>0</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2381,6 +3358,14 @@
           <t>Sold Out</t>
         </is>
       </c>
+      <c r="D49" t="b">
+        <v>0</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2396,6 +3381,14 @@
       <c r="C50" t="inlineStr">
         <is>
           <t>Sold Out</t>
+        </is>
+      </c>
+      <c r="D50" t="b">
+        <v>0</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>tier 0</t>
         </is>
       </c>
     </row>
@@ -2410,7 +3403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2429,6 +3422,16 @@
           <t>price</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>climate_controlled</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2446,6 +3449,14 @@
           <t>79.00</t>
         </is>
       </c>
+      <c r="D2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2463,6 +3474,14 @@
           <t>99.00</t>
         </is>
       </c>
+      <c r="D3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2480,6 +3499,14 @@
           <t>117.00</t>
         </is>
       </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>tier 1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2497,6 +3524,14 @@
           <t>175.00</t>
         </is>
       </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2514,6 +3549,14 @@
           <t>190.00</t>
         </is>
       </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>tier 1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2531,6 +3574,14 @@
           <t>270.00</t>
         </is>
       </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>tier 1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2548,6 +3599,14 @@
           <t>375.00</t>
         </is>
       </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2565,6 +3624,14 @@
           <t>450.00</t>
         </is>
       </c>
+      <c r="D9" t="b">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2582,6 +3649,14 @@
           <t>500.00</t>
         </is>
       </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>tier 1</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2599,6 +3674,14 @@
           <t>575.00</t>
         </is>
       </c>
+      <c r="D11" t="b">
+        <v>0</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2616,6 +3699,14 @@
           <t>695.00</t>
         </is>
       </c>
+      <c r="D12" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2633,6 +3724,14 @@
           <t>760.00</t>
         </is>
       </c>
+      <c r="D13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2650,6 +3749,14 @@
           <t>750.00</t>
         </is>
       </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2667,6 +3774,14 @@
           <t>199.00</t>
         </is>
       </c>
+      <c r="D15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2684,6 +3799,14 @@
           <t>299.00</t>
         </is>
       </c>
+      <c r="D16" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2701,6 +3824,14 @@
           <t>579.00</t>
         </is>
       </c>
+      <c r="D17" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2718,6 +3849,14 @@
           <t>650.00</t>
         </is>
       </c>
+      <c r="D18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2735,6 +3874,14 @@
           <t>1,300.00</t>
         </is>
       </c>
+      <c r="D19" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2752,6 +3899,14 @@
           <t>1,737.00</t>
         </is>
       </c>
+      <c r="D20" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2769,6 +3924,14 @@
           <t>299.00</t>
         </is>
       </c>
+      <c r="D21" t="b">
+        <v>0</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2786,6 +3949,14 @@
           <t>579.00</t>
         </is>
       </c>
+      <c r="D22" t="b">
+        <v>0</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2803,6 +3974,14 @@
           <t>650.00</t>
         </is>
       </c>
+      <c r="D23" t="b">
+        <v>0</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2818,6 +3997,14 @@
       <c r="C24" t="inlineStr">
         <is>
           <t>725.00</t>
+        </is>
+      </c>
+      <c r="D24" t="b">
+        <v>0</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>tier 3</t>
         </is>
       </c>
     </row>
@@ -2832,7 +4019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2851,6 +4038,16 @@
           <t>price</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>climate_controlled</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2868,6 +4065,14 @@
           <t>365.00</t>
         </is>
       </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2885,6 +4090,14 @@
           <t>199.00</t>
         </is>
       </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2902,6 +4115,14 @@
           <t>199.00</t>
         </is>
       </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2919,6 +4140,14 @@
           <t>260.00</t>
         </is>
       </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2936,6 +4165,14 @@
           <t>240.00</t>
         </is>
       </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2953,6 +4190,14 @@
           <t>305.00</t>
         </is>
       </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2970,6 +4215,14 @@
           <t>365.00</t>
         </is>
       </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2987,6 +4240,14 @@
           <t>405.00</t>
         </is>
       </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3004,6 +4265,14 @@
           <t>475.00</t>
         </is>
       </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3021,6 +4290,14 @@
           <t>450.00</t>
         </is>
       </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3038,6 +4315,14 @@
           <t>385.00</t>
         </is>
       </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3055,6 +4340,14 @@
           <t>440.00</t>
         </is>
       </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3072,6 +4365,14 @@
           <t>570.00</t>
         </is>
       </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3089,6 +4390,14 @@
           <t>470.00</t>
         </is>
       </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3106,6 +4415,14 @@
           <t>440.00</t>
         </is>
       </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3123,6 +4440,14 @@
           <t>440.00</t>
         </is>
       </c>
+      <c r="D17" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3140,6 +4465,14 @@
           <t>530.00</t>
         </is>
       </c>
+      <c r="D18" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3157,6 +4490,14 @@
           <t>50.00</t>
         </is>
       </c>
+      <c r="D19" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3174,6 +4515,14 @@
           <t>80.00</t>
         </is>
       </c>
+      <c r="D20" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3191,6 +4540,14 @@
           <t>85.00</t>
         </is>
       </c>
+      <c r="D21" t="b">
+        <v>0</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3208,6 +4565,14 @@
           <t>90.00</t>
         </is>
       </c>
+      <c r="D22" t="b">
+        <v>0</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3225,6 +4590,14 @@
           <t>165.00</t>
         </is>
       </c>
+      <c r="D23" t="b">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3234,12 +4607,20 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Climate Control- Indoor Access</t>
+          <t>Drive up access</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>175.00</t>
+        </is>
+      </c>
+      <c r="D24" t="b">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>tier 3</t>
         </is>
       </c>
     </row>
@@ -3251,12 +4632,20 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Drive up access</t>
+          <t>Climate Control- Indoor Access</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>175.00</t>
+        </is>
+      </c>
+      <c r="D25" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>tier 2</t>
         </is>
       </c>
     </row>
@@ -3276,6 +4665,14 @@
           <t>260.00</t>
         </is>
       </c>
+      <c r="D26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3293,6 +4690,14 @@
           <t>110.00</t>
         </is>
       </c>
+      <c r="D27" t="b">
+        <v>0</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3308,6 +4713,14 @@
       <c r="C28" t="inlineStr">
         <is>
           <t>145.00</t>
+        </is>
+      </c>
+      <c r="D28" t="b">
+        <v>0</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>tier 1</t>
         </is>
       </c>
     </row>
@@ -3322,7 +4735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3341,6 +4754,16 @@
           <t>price</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>climate_controlled</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3354,6 +4777,14 @@
           <t>44.00</t>
         </is>
       </c>
+      <c r="D2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3367,6 +4798,14 @@
           <t>96.00</t>
         </is>
       </c>
+      <c r="D3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3380,6 +4819,14 @@
           <t>320.00</t>
         </is>
       </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3397,6 +4844,14 @@
           <t>158.00</t>
         </is>
       </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>tier 0</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3414,6 +4869,14 @@
           <t>220.00</t>
         </is>
       </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>tier 1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3431,6 +4894,14 @@
           <t>110.00</t>
         </is>
       </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>tier 1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3448,6 +4919,14 @@
           <t>115.00</t>
         </is>
       </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3465,6 +4944,14 @@
           <t>120.00</t>
         </is>
       </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3482,6 +4969,14 @@
           <t>165.00</t>
         </is>
       </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>tier 1</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3499,6 +4994,14 @@
           <t>175.00</t>
         </is>
       </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3516,6 +5019,14 @@
           <t>185.00</t>
         </is>
       </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3533,6 +5044,14 @@
           <t>189.00</t>
         </is>
       </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>tier 1</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3550,6 +5069,14 @@
           <t>200.00</t>
         </is>
       </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>tier 2</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3567,6 +5094,14 @@
           <t>210.00</t>
         </is>
       </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>tier 3</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3582,6 +5117,14 @@
       <c r="C16" t="inlineStr">
         <is>
           <t>295.00</t>
+        </is>
+      </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>tier 3</t>
         </is>
       </c>
     </row>

</xml_diff>